<commit_message>
fix: close schedule import audit gaps
</commit_message>
<xml_diff>
--- a/tests/fixtures/automation/personal_schedule.xlsx
+++ b/tests/fixtures/automation/personal_schedule.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合成个人课表" sheetId="1" r:id="R6ed87fcdc9664d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无关页" sheetId="2" r:id="R319979a175c0483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合成个人课表" sheetId="1" r:id="R77721fd257ba4906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="无关页" sheetId="2" r:id="R0369c48f70184b27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -261,6 +261,7 @@
       <x:c r="D1"/>
       <x:c r="E1"/>
       <x:c r="F1"/>
+      <x:c r="G1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
@@ -273,12 +274,15 @@
         <x:v>课程名称</x:v>
       </x:c>
       <x:c r="D2" s="2" t="str">
+        <x:v>学年学期</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="str">
         <x:v>教学周</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="str">
+      <x:c r="F2" s="2" t="str">
         <x:v>星期几</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="str">
+      <x:c r="G2" s="2" t="str">
         <x:v>第几节</x:v>
       </x:c>
     </x:row>
@@ -291,12 +295,15 @@
         <x:v>合成课程甲</x:v>
       </x:c>
       <x:c r="D3" s="3" t="str">
+        <x:v>2026-synthetic-spring</x:v>
+      </x:c>
+      <x:c r="E3" s="3" t="str">
         <x:v>1-16周(双)</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="F3" s="3" t="str">
         <x:v>星期一</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="G3" s="3" t="str">
         <x:v>1-2节</x:v>
       </x:c>
     </x:row>
@@ -309,12 +316,15 @@
         <x:v>合成课程甲</x:v>
       </x:c>
       <x:c r="D4" s="3" t="str">
+        <x:v>2026-synthetic-spring</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="str">
         <x:v>1-16周(双)</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="F4" s="3" t="str">
         <x:v>星期一</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="G4" s="3" t="str">
         <x:v>1-2节</x:v>
       </x:c>
     </x:row>
@@ -327,22 +337,38 @@
         <x:v>合成课程乙</x:v>
       </x:c>
       <x:c r="D5" s="3" t="str">
+        <x:v>2026-synthetic-spring</x:v>
+      </x:c>
+      <x:c r="E5" s="3" t="str">
         <x:v>3-12周</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str">
+      <x:c r="F5" s="3" t="str">
         <x:v>周三</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="str">
+      <x:c r="G5" s="3" t="str">
         <x:v>5-6节</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="3"/>
+      <x:c r="A6" s="3" t="str">
+        <x:v>SYN-L-001</x:v>
+      </x:c>
       <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-      <x:c r="F6" s="3"/>
+      <x:c r="C6" s="3" t="str">
+        <x:v>合成错学期课程</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="str">
+        <x:v>2026-other-spring</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="str">
+        <x:v>2周</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="str">
+        <x:v>星期一</x:v>
+      </x:c>
+      <x:c r="G6" s="3" t="str">
+        <x:v>1-2节</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>